<commit_message>
Añadidos nuevos tickers. Creo que falta mejorarlos porque de algunos no encuentra información
</commit_message>
<xml_diff>
--- a/bolsa_resumen_auto.xlsx
+++ b/bolsa_resumen_auto.xlsx
@@ -340,10 +340,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.43359375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
+    <col width="17" customWidth="1" style="2" min="1" max="1"/>
     <col width="9" customWidth="1" style="2" min="2" max="3"/>
     <col width="9" customWidth="1" style="3" min="3" max="3"/>
     <col width="12" customWidth="1" style="2" min="4" max="4"/>
@@ -454,22 +454,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>€18,78</t>
+          <t>€18,81</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.59%</t>
+          <t>0.72%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6.49%</t>
+          <t>6.63%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>19.24%</t>
+          <t>19.40%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -526,22 +526,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>€62,70</t>
+          <t>€63,22</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>-31.11%</t>
+          <t>-30.54%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -598,22 +598,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>$273.54</t>
+          <t>$273.43</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>-1.45%</t>
+          <t>-1.48%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -650,19 +650,15 @@
     <row r="5" ht="15" customHeight="1" s="3">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OHLA</t>
+          <t>Telefónica</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OHLA.MC</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>BME</t>
-        </is>
-      </c>
+          <t>TEF</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>25/02/2026</t>
@@ -670,47 +666,47 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>€0,37</t>
+          <t>$4.27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-1.33%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-3.01%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>-13.25%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>€0,35</t>
+          <t>$3.75</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>€0,27</t>
+          <t>$3.67</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>€0,39</t>
+          <t>$4.46</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>€0,54</t>
+          <t>$5.72</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>€18,80</t>
+          <t>$34.50</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -722,19 +718,15 @@
     <row r="6" ht="15" customHeight="1" s="3">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Atos</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ATO.PA</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>EPA</t>
-        </is>
-      </c>
+          <t>SAN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>25/02/2026</t>
@@ -742,47 +734,47 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>€35,19</t>
+          <t>$13.02</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.03%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-15.42%</t>
+          <t>3.87%</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>-22.16%</t>
+          <t>21.86%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>€33,99</t>
+          <t>$11.74</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>€25,00</t>
+          <t>$5.54</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>€61,95</t>
+          <t>$13.19</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>€63,24</t>
+          <t>$13.19</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>€17.300,00</t>
+          <t>$22.34</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -794,67 +786,31 @@
     <row r="7" ht="15" customHeight="1" s="3">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alten</t>
+          <t>Banco Sabadell</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ATE.PA</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>EPA</t>
-        </is>
-      </c>
+          <t>SAB</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>25/02/2026</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>€59,55</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.85%</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>-0.92%</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>-11.78%</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>€55,55</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>€55,55</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>€84,00</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>€104,80</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>€163,30</t>
+          <t>$25.74</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -866,19 +822,15 @@
     <row r="8" ht="15" customHeight="1" s="3">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sopra Steria</t>
+          <t>BBVA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SOP.PA</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>EPA</t>
-        </is>
-      </c>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>25/02/2026</t>
@@ -886,47 +838,47 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>€121,40</t>
+          <t>$23.61</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.66%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>-8.03%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>€114,80</t>
+          <t>$22.50</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>€114,80</t>
+          <t>$11.59</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>€154,90</t>
+          <t>$26.20</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>€210,60</t>
+          <t>$26.20</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>€239,60</t>
+          <t>$26.20</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -938,12 +890,12 @@
     <row r="9" ht="15" customHeight="1" s="3">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>OHLA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IDR.MC</t>
+          <t>OHLA.MC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -958,47 +910,47 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>€50,85</t>
+          <t>€0,37</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-1.07%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-2.75%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>-13.01%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>€45,34</t>
+          <t>€0,35</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>€18,53</t>
+          <t>€0,27</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>€55,70</t>
+          <t>€0,39</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>€61,50</t>
+          <t>€0,54</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>€61,50</t>
+          <t>€18,80</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1010,1036 +962,2358 @@
     <row r="10" ht="15" customHeight="1" s="3">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Inditex (Zara)</t>
+          <t>Sacyr</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ITX.MC</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>BME</t>
-        </is>
-      </c>
+          <t>SYV</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>25/02/2026</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>€56,72</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>-1.43%</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>-1.80%</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>18.04%</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>€53,82</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>€40,80</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>€58,28</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>€58,28</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>€58,28</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
+          <t>$79.21</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="3">
       <c r="A11" t="inlineStr">
         <is>
+          <t>AENA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AENA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Acciona</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>$1.30</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ferrovial</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FER</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>$72.27</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-0.97%</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-1.43%</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>9.88%</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>$67.02</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>$40.46</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>$74.79</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>$74.79</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>$74.79</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Atos</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ATO.PA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EPA</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>€35,35</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-0.58%</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-15.04%</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>-21.80%</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>€33,99</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>€25,00</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>€61,95</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>€63,24</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>€17.300,00</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Alten</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ATE.PA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EPA</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>€59,80</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1.27%</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-0.50%</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>-11.41%</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>€55,55</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>€55,55</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>€84,00</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>€104,80</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>€163,30</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sopra Steria</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SOP.PA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>EPA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>€122,10</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3.12%</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1.24%</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>-7.50%</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>€114,80</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>€114,80</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>€154,90</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>€210,60</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>€239,60</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Indra</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IDR.MC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>€50,85</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>8.89%</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>€45,34</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>€18,53</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>€55,70</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>€61,50</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>€61,50</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Amadeus</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>$2.14</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>-1.38%</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-1.83%</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1.42%</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>$2.08</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>$2.01</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>$2.39</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>$3.11</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>$12.12</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Grifols</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>GRF</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>$10.70</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-1.83%</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.47%</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>8.08%</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>$10.36</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>$8.86</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>$11.32</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>$11.85</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>$12.00</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Inditex (Zara)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ITX.MC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>€56,72</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-1.43%</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-1.80%</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>18.04%</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>€53,82</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>€40,80</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>€58,28</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>€58,28</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>€58,28</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>YPF</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>YPF</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>NYSE</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>$37.30</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-1.87%</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-0.21%</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>3.44%</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>$36.04</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>$22.82</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>$40.38</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>$40.38</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>$69.98</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Iberdrola</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>IBE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>$10.39</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Repsol</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>REP.MC</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>€18,78</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>0.59%</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>6.49%</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>19.24%</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>€15,73</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>€9,41</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>€18,83</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>€18,83</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>€30,59</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Wolters Kluwer</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>WKL.AS</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>€62,70</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>0.80%</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>1.55%</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>-31.11%</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>€59,00</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>€59,00</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>€84,90</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>€172,65</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>€181,30</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>$273.54</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>0.51%</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>3.47%</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>-1.45%</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>$249.80</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>$169.21</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>$280.91</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>$288.62</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>$288.62</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>OHLA</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>OHLA.MC</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>€0,37</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>-1.33%</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>-3.01%</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>-13.25%</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>€0,35</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>€0,27</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>€0,39</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>€0,54</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>€18,80</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Atos</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>ATO.PA</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>EPA</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>€35,19</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>-1.03%</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>-15.42%</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>-22.16%</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>€33,99</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>€25,00</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>€61,95</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>€63,24</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>€17.300,00</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Alten</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>ATE.PA</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>EPA</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>€59,55</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>0.85%</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>-0.92%</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>-11.78%</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>€55,55</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>€55,55</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>€84,00</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>€104,80</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>€163,30</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Sopra Steria</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>SOP.PA</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>EPA</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>€121,40</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>2.53%</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>-8.03%</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>€114,80</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>€114,80</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>€154,90</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>€210,60</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>€239,60</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Indra</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>IDR.MC</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>€50,85</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>8.89%</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>€45,34</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>€18,53</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>€55,70</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>€61,50</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>€61,50</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Inditex (Zara)</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>ITX.MC</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>€56,72</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>-1.43%</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>-1.80%</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>18.04%</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>€53,82</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>€40,80</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>€58,28</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>€58,28</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>€58,28</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="3">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>YPF</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>YPF</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>$37.20</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>-2.13%</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>-0.48%</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>3.16%</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>$36.04</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>$22.82</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>$40.38</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>$40.38</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>$69.98</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="3">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Repsol</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>REP.MC</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>BME</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>€18,78</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>0.59%</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>6.49%</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>19.24%</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>€15,73</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>€9,41</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>€18,83</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>€18,83</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>€30,59</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="3">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Wolters Kluwer</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>WKL.AS</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>AMS</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>€62,74</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>0.87%</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>1.62%</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>-31.07%</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>€59,00</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>€59,00</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>€84,90</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>€172,65</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>€181,30</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="3">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Apple</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>$273.77</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>0.60%</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>3.57%</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>-1.36%</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>$249.80</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>$169.21</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>$280.91</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>$288.62</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>$288.62</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="3">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>OHLA</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>OHLA.MC</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>BME</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>€0,37</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>-1.47%</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>-3.15%</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>-13.36%</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>€0,35</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>€0,27</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>€0,39</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>€0,54</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>€18,80</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="3">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Atos</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>ATO.PA</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>EPA</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>€35,17</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>-1.05%</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>-15.44%</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>-22.18%</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>€33,99</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>€25,00</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>€61,95</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>€63,24</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>€17.300,00</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1" s="3">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Alten</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>ATE.PA</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>EPA</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>€59,40</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>0.59%</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>-1.16%</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>-12.00%</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>€55,55</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>€55,55</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>€84,00</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>€104,80</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>€163,30</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="3">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Sopra Steria</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>SOP.PA</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>EPA</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>€121,40</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>2.53%</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>0.66%</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>-8.03%</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>€114,80</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>€114,80</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>€154,90</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>€210,60</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>€239,60</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1" s="3">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Indra</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>IDR.MC</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>BME</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>€50,90</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>0.10%</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>-4.68%</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>8.99%</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>€45,34</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>€18,53</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>€55,70</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>€61,50</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>€61,50</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="3">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Inditex (Zara)</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>ITX.MC</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>BME</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>€56,76</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>-1.36%</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>-1.73%</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>18.13%</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>€53,82</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>€40,80</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>€58,28</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>€58,28</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>€58,28</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>YPF</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>YPF</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>NYSE</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>25/02/2026</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>$37.24</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>-2.03%</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>-0.37%</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>3.27%</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>$36.04</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>$22.82</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>$40.38</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>$40.38</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>$69.98</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (, )</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="3"/>
-    <row r="33" ht="15" customHeight="1" s="3"/>
-    <row r="34" ht="15" customHeight="1" s="3"/>
-    <row r="35" ht="15" customHeight="1" s="3"/>
-    <row r="36" ht="15" customHeight="1" s="3"/>
-    <row r="37" ht="15" customHeight="1" s="3"/>
-    <row r="38" ht="15" customHeight="1" s="3"/>
-    <row r="39" ht="15" customHeight="1" s="3"/>
-    <row r="40" ht="15" customHeight="1" s="3"/>
-    <row r="41" ht="15" customHeight="1" s="3"/>
-    <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
-      <c r="J42" s="2" t="n"/>
-      <c r="K42" s="2" t="n"/>
-      <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="n"/>
-      <c r="N42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
-      <c r="J43" s="2" t="n"/>
-      <c r="K43" s="2" t="n"/>
-      <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="n"/>
-      <c r="N43" s="2" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
-      <c r="J44" s="2" t="n"/>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
-      <c r="M44" s="2" t="n"/>
-      <c r="N44" s="2" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
-      <c r="J45" s="2" t="n"/>
-      <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="n"/>
-      <c r="M45" s="2" t="n"/>
-      <c r="N45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="n"/>
-      <c r="J46" s="2" t="n"/>
-      <c r="K46" s="2" t="n"/>
-      <c r="L46" s="2" t="n"/>
-      <c r="M46" s="2" t="n"/>
-      <c r="N46" s="2" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
-      <c r="J47" s="2" t="n"/>
-      <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="n"/>
-      <c r="N47" s="2" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
-      <c r="J48" s="2" t="n"/>
-      <c r="K48" s="2" t="n"/>
-      <c r="L48" s="2" t="n"/>
-      <c r="M48" s="2" t="n"/>
-      <c r="N48" s="2" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
-      <c r="G49" s="2" t="n"/>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="n"/>
-      <c r="J49" s="2" t="n"/>
-      <c r="K49" s="2" t="n"/>
-      <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="n"/>
-      <c r="N49" s="2" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
-      <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="n"/>
-      <c r="J50" s="2" t="n"/>
-      <c r="K50" s="2" t="n"/>
-      <c r="L50" s="2" t="n"/>
-      <c r="M50" s="2" t="n"/>
-      <c r="N50" s="2" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
-      <c r="J51" s="2" t="n"/>
-      <c r="K51" s="2" t="n"/>
-      <c r="L51" s="2" t="n"/>
-      <c r="M51" s="2" t="n"/>
-      <c r="N51" s="2" t="n"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (, )</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="n"/>
+      <c r="H63" s="2" t="n"/>
+      <c r="I63" s="2" t="n"/>
+      <c r="J63" s="2" t="n"/>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
+      <c r="M63" s="2" t="n"/>
+      <c r="N63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="n"/>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="2" t="n"/>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
+      <c r="M64" s="2" t="n"/>
+      <c r="N64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="n"/>
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
+      <c r="M65" s="2" t="n"/>
+      <c r="N65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="2" t="n"/>
+      <c r="G66" s="2" t="n"/>
+      <c r="H66" s="2" t="n"/>
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" s="2" t="n"/>
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" s="2" t="n"/>
+      <c r="M66" s="2" t="n"/>
+      <c r="N66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="n"/>
+      <c r="I67" s="2" t="n"/>
+      <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="n"/>
+      <c r="M67" s="2" t="n"/>
+      <c r="N67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="n"/>
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="n"/>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
+      <c r="M68" s="2" t="n"/>
+      <c r="N68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
+      <c r="M69" s="2" t="n"/>
+      <c r="N69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="n"/>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
+      <c r="M70" s="2" t="n"/>
+      <c r="N70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="n"/>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="n"/>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
+      <c r="M71" s="2" t="n"/>
+      <c r="N71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="n"/>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="n"/>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="n"/>
+      <c r="M72" s="2" t="n"/>
+      <c r="N72" s="2" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>